<commit_message>
Fix field mapping in exam schedule database to populate all grade posters and filters
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -3475,7 +3475,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Grade  6</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -11787,7 +11787,7 @@
         </is>
       </c>
       <c r="L203" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="204">
@@ -11819,7 +11819,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -11843,7 +11843,7 @@
         </is>
       </c>
       <c r="L204" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="205">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="L205" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="206">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -11955,7 +11955,7 @@
         </is>
       </c>
       <c r="L206" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="207">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>Kinder 1</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -12011,7 +12011,7 @@
         </is>
       </c>
       <c r="L207" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="208">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>Kinder 1</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -12067,7 +12067,7 @@
         </is>
       </c>
       <c r="L208" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="209">
@@ -12099,7 +12099,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>Kinder 1</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -12123,7 +12123,7 @@
         </is>
       </c>
       <c r="L209" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="210">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>Kinder 1</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -12179,7 +12179,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="211">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -15315,7 +15315,7 @@
         </is>
       </c>
       <c r="L266" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="267">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -15371,7 +15371,7 @@
         </is>
       </c>
       <c r="L267" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="268">
@@ -15403,7 +15403,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -15427,7 +15427,7 @@
         </is>
       </c>
       <c r="L268" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="269">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -15483,7 +15483,7 @@
         </is>
       </c>
       <c r="L269" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="270">

</xml_diff>

<commit_message>
fix: accommodate Teacher Sophia exam duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -28054,22 +28054,22 @@
       </c>
       <c r="J419" t="inlineStr">
         <is>
-          <t>subj_mapeh</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t>MAPEH</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="N419" t="n">
@@ -37558,22 +37558,22 @@
       </c>
       <c r="J563" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_mapeh</t>
         </is>
       </c>
       <c r="K563" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>MAPEH</t>
         </is>
       </c>
       <c r="L563" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="M563" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Teacher Franchette</t>
         </is>
       </c>
       <c r="N563" t="n">

</xml_diff>

<commit_message>
fix: adjust elementary GMRC exam slots
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -2685,12 +2685,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2710,22 +2710,22 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>tchr_saliha</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Ustadha Saliha</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="N35" t="n">
@@ -2751,12 +2751,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
+          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
+          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2776,22 +2776,22 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_silfah</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Ustadh Silfah</t>
         </is>
       </c>
       <c r="N36" t="n">
@@ -2808,21 +2808,21 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>11:30 AM – 12:30 PM</t>
+          <t>12:40 PM – 01:40 PM</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
+          <t>sec_grade_1_ali_ibn_abi_talib_1st_shift</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
+          <t>GRADE 1 - ALI IBN ABI TALIB(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Grade 6</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2842,22 +2842,22 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_makabansa</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Makabansa</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>tchr_silfah</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Ustadh Silfah</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N37" t="n">
@@ -2883,12 +2883,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>sec_grade_1_ali_ibn_abi_talib_1st_shift</t>
+          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>GRADE 1 - ALI IBN ABI TALIB(1ST SHIFT)</t>
+          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2908,22 +2908,22 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>subj_makabansa</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Makabansa</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N38" t="n">
@@ -2949,22 +2949,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
+          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
+          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2974,22 +2974,22 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_social_studies</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Social Science</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="N39" t="n">
@@ -3006,7 +3006,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3015,22 +3015,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3040,22 +3040,22 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>subj_social_studies</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Social Science</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_abdulwahab</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Alim Abdulwahab</t>
         </is>
       </c>
       <c r="N40" t="n">
@@ -3081,12 +3081,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3106,22 +3106,22 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_pe_12</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>PE 12</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="N41" t="n">
@@ -3138,7 +3138,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3147,22 +3147,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3172,22 +3172,22 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>subj_pe_12</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>PE 12</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_abdul_karim</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Alim Abdul Karim</t>
         </is>
       </c>
       <c r="N42" t="n">
@@ -3213,12 +3213,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
+          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
+          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3238,22 +3238,22 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>tchr_abdul_karim</t>
+          <t>tchr_sitti_kauzar</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Alim Abdul Karim</t>
+          <t>Teacher Sitti Kauzar</t>
         </is>
       </c>
       <c r="N43" t="n">
@@ -3279,12 +3279,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3304,22 +3304,22 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>tchr_sitti_kauzar</t>
+          <t>tchr_obaydah</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Teacher Sitti Kauzar</t>
+          <t>Ustadh Obaydah</t>
         </is>
       </c>
       <c r="N44" t="n">
@@ -3345,12 +3345,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3370,22 +3370,22 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>tchr_obaydah</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Ustadh Obaydah</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N45" t="n">
@@ -3411,12 +3411,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3436,22 +3436,22 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_anna</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Anna</t>
         </is>
       </c>
       <c r="N46" t="n">
@@ -3477,12 +3477,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3502,22 +3502,22 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>tchr_anna</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Teacher Anna</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N47" t="n">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3568,22 +3568,22 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_saliha</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Ustadha Saliha</t>
         </is>
       </c>
       <c r="N48" t="n">
@@ -4062,21 +4062,21 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>01:30 PM – 02:30 PM</t>
+          <t>01:50 PM – 02:50 PM</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>sec_kinder_2_uthman_ibn_affan_1st_shift</t>
+          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Kinder 2 UTHMAN IBN AFFAN (1ST SHIFT)</t>
+          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Kinder 2</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4096,22 +4096,22 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>subj_hadith</t>
+          <t>subj_makabansa</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Hadith</t>
+          <t>Makabansa</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>tchr_saliha</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Ustadha Saliha</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N56" t="n">
@@ -4137,22 +4137,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
+          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
+          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4162,22 +4162,22 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>subj_makabansa</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Makabansa</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_abdulwahab</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Alim Abdulwahab</t>
         </is>
       </c>
       <c r="N57" t="n">
@@ -4194,7 +4194,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4203,22 +4203,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4228,22 +4228,22 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -4269,12 +4269,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4294,22 +4294,22 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_gen_bio_1</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Gen Bio 1</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_radzmia</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Teacher Radzmia</t>
         </is>
       </c>
       <c r="N59" t="n">
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4335,22 +4335,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4360,22 +4360,22 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>subj_gen_bio_1</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Gen Bio 1</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>tchr_radzmia</t>
+          <t>tchr_sitti_kauzar</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Teacher Radzmia</t>
+          <t>Teacher Sitti Kauzar</t>
         </is>
       </c>
       <c r="N60" t="n">
@@ -4401,12 +4401,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
+          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
+          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4426,22 +4426,22 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_makabansa</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Makabansa</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>tchr_sitti_kauzar</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Teacher Sitti Kauzar</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N61" t="n">
@@ -4458,7 +4458,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -4467,12 +4467,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
+          <t>sec_grade_3_as_ad_ibn_zurarah_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
+          <t>GRADE 3 - AS'AD IBN ZURARAH (2ND SHIFT) MIX</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -4482,32 +4482,32 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>subj_makabansa</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Makabansa</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_saliha</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Ustadha Saliha</t>
         </is>
       </c>
       <c r="N62" t="n">
@@ -15216,21 +15216,21 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>03:10 PM – 04:10 PM</t>
+          <t>02:40 PM – 03:40 PM</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
+          <t>sec_kinder_2_uthman_ibn_affan_1st_shift</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
+          <t>Kinder 2 UTHMAN IBN AFFAN (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -15240,7 +15240,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -15250,22 +15250,22 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_hadith</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Hadith</t>
         </is>
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>tchr_joanna</t>
+          <t>tchr_saliha</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>Teacher Joanna</t>
+          <t>Ustadha Saliha</t>
         </is>
       </c>
       <c r="N225" t="n">
@@ -15282,7 +15282,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D226" t="inlineStr">
         <is>
@@ -15291,12 +15291,12 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
+          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
+          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -15311,27 +15311,27 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_joanna</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Teacher Joanna</t>
         </is>
       </c>
       <c r="N226" t="n">
@@ -15357,12 +15357,12 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>sec_grade_1_suhayb_ar_rumi_2nd_shift</t>
+          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>GRADE 1 - SUHAYB AR-RUMI (2ND SHIFT)</t>
+          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -15382,22 +15382,22 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>subj_language</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N227" t="n">
@@ -15423,22 +15423,22 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
+          <t>sec_grade_1_suhayb_ar_rumi_2nd_shift</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
+          <t>GRADE 1 - SUHAYB AR-RUMI (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15448,22 +15448,22 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_language</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N228" t="n">
@@ -15480,7 +15480,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -15489,12 +15489,12 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
+          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
+          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -15509,27 +15509,27 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>tchr_norhaima</t>
+          <t>tchr_abdulwahab</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>Teacher Norhaima</t>
+          <t>Alim Abdulwahab</t>
         </is>
       </c>
       <c r="N229" t="n">
@@ -15546,7 +15546,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D230" t="inlineStr">
         <is>
@@ -15555,47 +15555,47 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>sec_grade_11_2nd_shift_boys</t>
+          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>GRADE 11 (2ND SHIFT BOYS)</t>
+          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>subj_mabisang_komunikasyon</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>Mabisang Komunikasyon</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_norhaima</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Teacher Norhaima</t>
         </is>
       </c>
       <c r="N230" t="n">
@@ -15621,22 +15621,22 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
+          <t>sec_grade_11_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
+          <t>GRADE 11 (2ND SHIFT BOYS)</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15646,22 +15646,22 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_mabisang_komunikasyon</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Mabisang Komunikasyon</t>
         </is>
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N231" t="n">
@@ -15687,12 +15687,12 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>sec_grade_3_as_ad_ibn_zurarah_2nd_shift_mix</t>
+          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>GRADE 3 - AS'AD IBN ZURARAH (2ND SHIFT) MIX</t>
+          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -15702,7 +15702,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15712,22 +15712,22 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>tchr_saliha</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>Ustadha Saliha</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N232" t="n">

</xml_diff>

<commit_message>
fix: remove duplicate SHS timetable cells
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -15942,7 +15942,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -15951,47 +15951,47 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_mil</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="N236" t="n">
@@ -16008,7 +16008,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -16017,12 +16017,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -16032,32 +16032,32 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>subj_fil3</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Fil3</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N237" t="n">
@@ -16074,7 +16074,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -16083,12 +16083,12 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -16103,27 +16103,27 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_fil3</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Fil3</t>
         </is>
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N238" t="n">
@@ -16149,12 +16149,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -16174,22 +16174,22 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="M239" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="N239" t="n">
@@ -16206,7 +16206,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D240" t="inlineStr">
         <is>
@@ -16215,12 +16215,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -16235,27 +16235,27 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N240" t="n">
@@ -16272,7 +16272,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -16281,12 +16281,12 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -16296,32 +16296,32 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="N241" t="n">
@@ -16338,7 +16338,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -16347,12 +16347,12 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -16367,27 +16367,27 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N242" t="n">
@@ -16404,7 +16404,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
@@ -16413,12 +16413,12 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -16433,27 +16433,27 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="N243" t="n">
@@ -16479,12 +16479,12 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -16504,22 +16504,22 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N244" t="n">
@@ -16536,7 +16536,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
@@ -16545,12 +16545,12 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -16560,32 +16560,32 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>tchr_faidh</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>Ustadh Faidh</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N245" t="n">
@@ -16611,12 +16611,12 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -16636,22 +16636,22 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>tchr_jairah</t>
+          <t>tchr_faidh</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>Teacher Jairah</t>
+          <t>Ustadh Faidh</t>
         </is>
       </c>
       <c r="N246" t="n">
@@ -16677,12 +16677,12 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
+          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
+          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -16702,22 +16702,22 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_jairah</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Jairah</t>
         </is>
       </c>
       <c r="N247" t="n">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -16743,12 +16743,12 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>sec_grade_5_mus_ab_ibn_abdul_mutalib_2nd_shift</t>
+          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUS'AB IBN ABDUL MUTALIB (2ND SHIFT)</t>
+          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -16763,27 +16763,27 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Teacher Keychell</t>
         </is>
       </c>
       <c r="N248" t="n">
@@ -16800,7 +16800,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -16809,12 +16809,12 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
+          <t>sec_grade_5_mus_ab_ibn_abdul_mutalib_2nd_shift</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
+          <t>GRADE 5 - MUS'AB IBN ABDUL MUTALIB (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -16824,32 +16824,32 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>Grade 6</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>tchr_jessa</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>Teacher Jessa</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="N249" t="n">
@@ -16866,7 +16866,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D250" t="inlineStr">
         <is>
@@ -16875,12 +16875,12 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>sec_grade_6_dihya_ibn_khalifah_2nd_shift_girls</t>
+          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>GRADE 6 - DIHYA IBN KHALIFAH (2ND SHIFT) GIRLS</t>
+          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -16895,27 +16895,27 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>tchr_obaydah</t>
+          <t>tchr_jessa</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Ustadh Obaydah</t>
+          <t>Teacher Jessa</t>
         </is>
       </c>
       <c r="N250" t="n">
@@ -16941,12 +16941,12 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
+          <t>sec_grade_6_dihya_ibn_khalifah_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
+          <t>GRADE 6 - DIHYA IBN KHALIFAH (2ND SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -16966,22 +16966,22 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_obaydah</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Ustadh Obaydah</t>
         </is>
       </c>
       <c r="N251" t="n">
@@ -16998,7 +16998,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D252" t="inlineStr">
         <is>
@@ -17007,47 +17007,47 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
+          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
+          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Grade 7</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>subj_social_studies</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>tchr_shirehan</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Teacher Shirehan</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N252" t="n">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D253" t="inlineStr">
         <is>
@@ -17073,12 +17073,12 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
+          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
+          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -17093,27 +17093,27 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_social_studies</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>tchr_silfah</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>Ustadh Silfah</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="N253" t="n">
@@ -17130,7 +17130,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D254" t="inlineStr">
         <is>
@@ -17139,12 +17139,12 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
+          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
+          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -17159,27 +17159,27 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>tchr_aniah</t>
+          <t>tchr_silfah</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>Teacher Aniah</t>
+          <t>Ustadh Silfah</t>
         </is>
       </c>
       <c r="N254" t="n">
@@ -17196,7 +17196,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D255" t="inlineStr">
         <is>
@@ -17205,12 +17205,12 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
+          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
+          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>Grade 8</t>
+          <t>Grade 7</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -17240,12 +17240,12 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>tchr_radzmia</t>
+          <t>tchr_aniah</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>Teacher Radzmia</t>
+          <t>Teacher Aniah</t>
         </is>
       </c>
       <c r="N255" t="n">
@@ -17271,12 +17271,12 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
+          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
+          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -17296,22 +17296,22 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>tchr_halnaisa</t>
+          <t>tchr_radzmia</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>Teacher Halnaisa</t>
+          <t>Teacher Radzmia</t>
         </is>
       </c>
       <c r="N256" t="n">
@@ -17328,7 +17328,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D257" t="inlineStr">
         <is>
@@ -17337,12 +17337,12 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
+          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -17357,27 +17357,27 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>tchr_samsuddin</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>Alim Samsuddin</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N257" t="n">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D258" t="inlineStr">
         <is>
@@ -17403,12 +17403,12 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
+          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
+          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -17418,32 +17418,32 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>Grade 9</t>
+          <t>Grade 8</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>subj_social_studies</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>Social Science</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_samsuddin</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Alim Samsuddin</t>
         </is>
       </c>
       <c r="N258" t="n">
@@ -17469,12 +17469,12 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_jandal_ibn_suhayl_2nd_shift_girls</t>
+          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU JANDAL IBN SUHAYL (2ND SHIFT) GIRLS</t>
+          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -17494,22 +17494,22 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_social_studies</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Social Science</t>
         </is>
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>tchr_angeleni</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>Teacher Angeleni</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="N259" t="n">
@@ -17526,21 +17526,21 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>04:20 PM – 05:20 PM</t>
+          <t>03:10 PM – 04:10 PM</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
+          <t>sec_grade_9_abu_jandal_ibn_suhayl_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
+          <t>GRADE 9 - ABU JANDAL IBN SUHAYL (2ND SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 9</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17560,22 +17560,22 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_angeleni</t>
         </is>
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Teacher Angeleni</t>
         </is>
       </c>
       <c r="N260" t="n">
@@ -17592,7 +17592,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -17601,47 +17601,47 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>subj_gen_bio_1</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Gen Bio 1</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N261" t="n">
@@ -17658,21 +17658,21 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>04:20 PM – 06:30 PM</t>
+          <t>04:20 PM – 05:20 PM</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>sec_grade_11_2nd_shift_boys</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>GRADE 11 (2ND SHIFT BOYS)</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -17687,31 +17687,31 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>subj_gen_math</t>
+          <t>subj_gen_bio_1</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>Gen Math</t>
+          <t>Gen Bio 1</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>tchr_jhelyn</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>Teacher Jhelyn</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="N262" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="263">
@@ -17724,21 +17724,21 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>04:20 PM – 05:20 PM</t>
+          <t>04:20 PM – 06:30 PM</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_11_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 11 (2ND SHIFT BOYS)</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -17748,36 +17748,36 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>subj_mil</t>
+          <t>subj_gen_math</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>Gen Math</t>
         </is>
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_jhelyn</t>
         </is>
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Teacher Jhelyn</t>
         </is>
       </c>
       <c r="N263" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="264">
@@ -25512,7 +25512,7 @@
         </is>
       </c>
       <c r="C381" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D381" t="inlineStr">
         <is>
@@ -25521,47 +25521,47 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J381" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_prac_res_2</t>
         </is>
       </c>
       <c r="K381" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Prac. Res. 2</t>
         </is>
       </c>
       <c r="L381" t="inlineStr">
         <is>
-          <t>tchr_sitti_kauzar</t>
+          <t>tchr_aniah</t>
         </is>
       </c>
       <c r="M381" t="inlineStr">
         <is>
-          <t>Teacher Sitti Kauzar</t>
+          <t>Teacher Aniah</t>
         </is>
       </c>
       <c r="N381" t="n">
@@ -25587,12 +25587,12 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>sec_grade_3_as_ad_ibn_zurarah_2nd_shift_mix</t>
+          <t>sec_grade_2_saeed_ibn_zayd_2nd_shift</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>GRADE 3 - AS'AD IBN ZURARAH (2ND SHIFT) MIX</t>
+          <t>GRADE 2 - SAEED IBN ZAYD (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -25602,7 +25602,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -25612,22 +25612,22 @@
       </c>
       <c r="J382" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">
         <is>
-          <t>tchr_faidh</t>
+          <t>tchr_sitti_kauzar</t>
         </is>
       </c>
       <c r="M382" t="inlineStr">
         <is>
-          <t>Ustadh Faidh</t>
+          <t>Teacher Sitti Kauzar</t>
         </is>
       </c>
       <c r="N382" t="n">
@@ -25644,7 +25644,7 @@
         </is>
       </c>
       <c r="C383" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D383" t="inlineStr">
         <is>
@@ -25653,12 +25653,12 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
+          <t>sec_grade_3_as_ad_ibn_zurarah_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 3 - AS'AD IBN ZURARAH (2ND SHIFT) MIX</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
@@ -25673,27 +25673,27 @@
       </c>
       <c r="I383" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J383" t="inlineStr">
         <is>
-          <t>subj_makabansa</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
         <is>
-          <t>Makabansa</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L383" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_faidh</t>
         </is>
       </c>
       <c r="M383" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Ustadh Faidh</t>
         </is>
       </c>
       <c r="N383" t="n">
@@ -25719,12 +25719,12 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
@@ -25744,22 +25744,22 @@
       </c>
       <c r="J384" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_makabansa</t>
         </is>
       </c>
       <c r="K384" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Makabansa</t>
         </is>
       </c>
       <c r="L384" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_zara</t>
         </is>
       </c>
       <c r="M384" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Zara</t>
         </is>
       </c>
       <c r="N384" t="n">
@@ -25776,7 +25776,7 @@
         </is>
       </c>
       <c r="C385" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D385" t="inlineStr">
         <is>
@@ -25785,12 +25785,12 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
@@ -25805,27 +25805,27 @@
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>tchr_normylah</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M385" t="inlineStr">
         <is>
-          <t>Teacher Normylah</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N385" t="n">
@@ -25842,7 +25842,7 @@
         </is>
       </c>
       <c r="C386" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D386" t="inlineStr">
         <is>
@@ -25851,12 +25851,12 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -25871,27 +25871,27 @@
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J386" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_normylah</t>
         </is>
       </c>
       <c r="M386" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Normylah</t>
         </is>
       </c>
       <c r="N386" t="n">
@@ -25917,12 +25917,12 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -25932,7 +25932,7 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I387" t="inlineStr">
@@ -25942,22 +25942,22 @@
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N387" t="n">
@@ -25974,7 +25974,7 @@
         </is>
       </c>
       <c r="C388" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
@@ -25983,12 +25983,12 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -26003,27 +26003,27 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N388" t="n">
@@ -26049,12 +26049,12 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -26074,22 +26074,22 @@
       </c>
       <c r="J389" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M389" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N389" t="n">
@@ -26106,7 +26106,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -26115,12 +26115,12 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -26135,27 +26135,27 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
         <is>
-          <t>subj_fil4</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>Fil4</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N390" t="n">
@@ -26172,7 +26172,7 @@
         </is>
       </c>
       <c r="C391" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D391" t="inlineStr">
         <is>
@@ -26181,12 +26181,12 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -26201,27 +26201,27 @@
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J391" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_fil4</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Fil4</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N391" t="n">
@@ -26247,12 +26247,12 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -26262,7 +26262,7 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
@@ -26272,22 +26272,22 @@
       </c>
       <c r="J392" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>tchr_fhairudz</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t>Teacher Fhairudz</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N392" t="n">
@@ -26304,7 +26304,7 @@
         </is>
       </c>
       <c r="C393" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -26313,12 +26313,12 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
+          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
+          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -26333,27 +26333,27 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t>tchr_jessa</t>
+          <t>tchr_fhairudz</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>Teacher Jessa</t>
+          <t>Teacher Fhairudz</t>
         </is>
       </c>
       <c r="N393" t="n">
@@ -26370,7 +26370,7 @@
         </is>
       </c>
       <c r="C394" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D394" t="inlineStr">
         <is>
@@ -26379,12 +26379,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>sec_grade_5_ja_far_ibn_abi_talib_2nd_shift_mix</t>
+          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>GRADE 5 - JA'FAR IBN ABI TALIB (2ND SHIFT) - MIX</t>
+          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -26399,27 +26399,27 @@
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J394" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
         <is>
-          <t>tchr_obaydah</t>
+          <t>tchr_jessa</t>
         </is>
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>Ustadh Obaydah</t>
+          <t>Teacher Jessa</t>
         </is>
       </c>
       <c r="N394" t="n">
@@ -26436,7 +26436,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -26445,12 +26445,12 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
+          <t>sec_grade_5_ja_far_ibn_abi_talib_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
+          <t>GRADE 5 - JA'FAR IBN ABI TALIB (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -26465,27 +26465,27 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
         <is>
-          <t>subj_mapeh</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t>MAPEH</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_obaydah</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Ustadh Obaydah</t>
         </is>
       </c>
       <c r="N395" t="n">
@@ -26502,7 +26502,7 @@
         </is>
       </c>
       <c r="C396" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D396" t="inlineStr">
         <is>
@@ -26511,12 +26511,12 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>sec_grade_5_mus_ab_ibn_abdul_mutalib_2nd_shift</t>
+          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUS'AB IBN ABDUL MUTALIB (2ND SHIFT)</t>
+          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
@@ -26531,27 +26531,27 @@
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J396" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_mapeh</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>MAPEH</t>
         </is>
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="M396" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Teacher Keychell</t>
         </is>
       </c>
       <c r="N396" t="n">
@@ -26568,7 +26568,7 @@
         </is>
       </c>
       <c r="C397" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D397" t="inlineStr">
         <is>
@@ -26577,12 +26577,12 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>sec_grade_6_abdullah_ibn_salaam_1st_shift</t>
+          <t>sec_grade_5_mus_ab_ibn_abdul_mutalib_2nd_shift</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABDULLAH IBN SALAAM (1ST SHIFT)</t>
+          <t>GRADE 5 - MUS'AB IBN ABDUL MUTALIB (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -26592,32 +26592,32 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>Grade 6</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="M397" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="N397" t="n">
@@ -26634,7 +26634,7 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
@@ -26643,12 +26643,12 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
+          <t>sec_grade_6_abdullah_ibn_salaam_1st_shift</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
+          <t>GRADE 6 - ABDULLAH IBN SALAAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -26663,27 +26663,27 @@
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J398" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M398" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N398" t="n">
@@ -26700,7 +26700,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -26709,47 +26709,47 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
+          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
+          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>Grade 7</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J399" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>tchr_samsuddin</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="M399" t="inlineStr">
         <is>
-          <t>Alim Samsuddin</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="N399" t="n">
@@ -26766,21 +26766,21 @@
         </is>
       </c>
       <c r="C400" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>03:10 PM – 05:20 PM</t>
+          <t>03:10 PM – 04:10 PM</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
+          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
+          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
@@ -26795,31 +26795,31 @@
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_samsuddin</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Alim Samsuddin</t>
         </is>
       </c>
       <c r="N400" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="401">
@@ -26832,21 +26832,21 @@
         </is>
       </c>
       <c r="C401" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>03:10 PM – 04:10 PM</t>
+          <t>03:10 PM – 05:20 PM</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
+          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
+          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -26861,31 +26861,31 @@
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t>tchr_jairah</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
         <is>
-          <t>Teacher Jairah</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="N401" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="402">
@@ -26898,7 +26898,7 @@
         </is>
       </c>
       <c r="C402" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D402" t="inlineStr">
         <is>
@@ -26907,12 +26907,12 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
+          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
+          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -26922,32 +26922,32 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>Grade 8</t>
+          <t>Grade 7</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J402" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_jairah</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Teacher Jairah</t>
         </is>
       </c>
       <c r="N402" t="n">
@@ -26973,12 +26973,12 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
+          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
+          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -26998,22 +26998,22 @@
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>subj_values_ed</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t>Values Ed</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="N403" t="n">
@@ -27030,7 +27030,7 @@
         </is>
       </c>
       <c r="C404" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D404" t="inlineStr">
         <is>
@@ -27039,12 +27039,12 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
+          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -27059,27 +27059,27 @@
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J404" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_values_ed</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Values Ed</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>tchr_radzmia</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
         <is>
-          <t>Teacher Radzmia</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="N404" t="n">
@@ -27096,21 +27096,21 @@
         </is>
       </c>
       <c r="C405" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>03:10 PM – 05:20 PM</t>
+          <t>03:10 PM – 04:10 PM</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
+          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
+          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -27120,36 +27120,36 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>Grade 9</t>
+          <t>Grade 8</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>tchr_jhelyn</t>
+          <t>tchr_radzmia</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
         <is>
-          <t>Teacher Jhelyn</t>
+          <t>Teacher Radzmia</t>
         </is>
       </c>
       <c r="N405" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="406">
@@ -27162,21 +27162,21 @@
         </is>
       </c>
       <c r="C406" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>03:10 PM – 04:10 PM</t>
+          <t>03:10 PM – 05:20 PM</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
+          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
+          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -27191,31 +27191,31 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_jhelyn</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Teacher Jhelyn</t>
         </is>
       </c>
       <c r="N406" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="407">
@@ -27228,7 +27228,7 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
@@ -27237,12 +27237,12 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_jandal_ibn_suhayl_2nd_shift_girls</t>
+          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU JANDAL IBN SUHAYL (2ND SHIFT) GIRLS</t>
+          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -27257,27 +27257,27 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>tchr_norhaima</t>
+          <t>tchr_abdulwahab</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
         <is>
-          <t>Teacher Norhaima</t>
+          <t>Alim Abdulwahab</t>
         </is>
       </c>
       <c r="N407" t="n">
@@ -27294,31 +27294,31 @@
         </is>
       </c>
       <c r="C408" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>04:20 PM – 05:20 PM</t>
+          <t>03:10 PM – 04:10 PM</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
+          <t>sec_grade_9_abu_jandal_ibn_suhayl_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
+          <t>GRADE 9 - ABU JANDAL IBN SUHAYL (2ND SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Grade 9</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
@@ -27328,22 +27328,22 @@
       </c>
       <c r="J408" t="inlineStr">
         <is>
-          <t>subj_language</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_norhaima</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Norhaima</t>
         </is>
       </c>
       <c r="N408" t="n">
@@ -27369,12 +27369,12 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>sec_grade_1_suhayb_ar_rumi_2nd_shift</t>
+          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>GRADE 1 - SUHAYB AR-RUMI (2ND SHIFT)</t>
+          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -27394,22 +27394,22 @@
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_language</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N409" t="n">
@@ -27435,22 +27435,22 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
+          <t>sec_grade_1_suhayb_ar_rumi_2nd_shift</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
+          <t>GRADE 1 - SUHAYB AR-RUMI (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
@@ -27460,22 +27460,22 @@
       </c>
       <c r="J410" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K410" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t>tchr_angeleni</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>Teacher Angeleni</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N410" t="n">
@@ -27492,7 +27492,7 @@
         </is>
       </c>
       <c r="C411" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D411" t="inlineStr">
         <is>
@@ -27501,47 +27501,47 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J411" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>tchr_samsuddin</t>
+          <t>tchr_angeleni</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>Alim Samsuddin</t>
+          <t>Teacher Angeleni</t>
         </is>
       </c>
       <c r="N411" t="n">
@@ -27558,7 +27558,7 @@
         </is>
       </c>
       <c r="C412" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D412" t="inlineStr">
         <is>
@@ -27567,12 +27567,12 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>sec_grade_11_2nd_shift_boys</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>GRADE 11 (2ND SHIFT BOYS)</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -27587,27 +27587,27 @@
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
         <is>
-          <t>subj_ec</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_samsuddin</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Samsuddin</t>
         </is>
       </c>
       <c r="N412" t="n">
@@ -27624,7 +27624,7 @@
         </is>
       </c>
       <c r="C413" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D413" t="inlineStr">
         <is>
@@ -27633,12 +27633,12 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_11_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 11 (2ND SHIFT BOYS)</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -27648,32 +27648,32 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
         <is>
-          <t>subj_prac_res_2</t>
+          <t>subj_ec</t>
         </is>
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t>Prac. Res. 2</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>tchr_aniah</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
         <is>
-          <t>Teacher Aniah</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N413" t="n">

</xml_diff>

<commit_message>
fix: correct Teacher Keychelle spelling
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -2395,7 +2395,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N30" t="n">
@@ -9325,7 +9325,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N135" t="n">
@@ -13615,7 +13615,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N200" t="n">
@@ -16783,7 +16783,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N248" t="n">
@@ -26551,7 +26551,7 @@
       </c>
       <c r="M396" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N396" t="n">
@@ -30643,7 +30643,7 @@
       </c>
       <c r="M458" t="inlineStr">
         <is>
-          <t>Teacher Keychell</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N458" t="n">

</xml_diff>

<commit_message>
fix: move Grade 11 Mabisang exam to Sunday
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -22419,12 +22419,12 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I334" t="inlineStr">
@@ -22444,22 +22444,22 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_mabisang_komunikasyon</t>
         </is>
       </c>
       <c r="K334" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Mabisang Komunikasyon</t>
         </is>
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>tchr_samsuddin</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
         <is>
-          <t>Alim Samsuddin</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N334" t="n">
@@ -22485,22 +22485,22 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
@@ -22510,22 +22510,22 @@
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t>tchr_sitti_kauzar</t>
+          <t>tchr_samsuddin</t>
         </is>
       </c>
       <c r="M335" t="inlineStr">
         <is>
-          <t>Teacher Sitti Kauzar</t>
+          <t>Alim Samsuddin</t>
         </is>
       </c>
       <c r="N335" t="n">
@@ -22551,12 +22551,12 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
+          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
+          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -22576,22 +22576,22 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>tchr_obaydah</t>
+          <t>tchr_sitti_kauzar</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
         <is>
-          <t>Ustadh Obaydah</t>
+          <t>Teacher Sitti Kauzar</t>
         </is>
       </c>
       <c r="N336" t="n">
@@ -22617,12 +22617,12 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
+          <t>sec_grade_2_talha_ibn_ubaydullah_1st_shift</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 2 - TALHA IBN UBAYDULLAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -22642,22 +22642,22 @@
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>tchr_silfah</t>
+          <t>tchr_obaydah</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t>Ustadh Silfah</t>
+          <t>Ustadh Obaydah</t>
         </is>
       </c>
       <c r="N337" t="n">
@@ -22683,12 +22683,12 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -22708,22 +22708,22 @@
       </c>
       <c r="J338" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_silfah</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Ustadh Silfah</t>
         </is>
       </c>
       <c r="N338" t="n">
@@ -22749,12 +22749,12 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -22774,22 +22774,22 @@
       </c>
       <c r="J339" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t>tchr_normylah</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="M339" t="inlineStr">
         <is>
-          <t>Teacher Normylah</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="N339" t="n">
@@ -22815,12 +22815,12 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -22830,7 +22830,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -22840,22 +22840,22 @@
       </c>
       <c r="J340" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_normylah</t>
         </is>
       </c>
       <c r="M340" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Normylah</t>
         </is>
       </c>
       <c r="N340" t="n">
@@ -22881,12 +22881,12 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -22906,22 +22906,22 @@
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M341" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N341" t="n">
@@ -22947,12 +22947,12 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -22972,22 +22972,22 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="N342" t="n">
@@ -23013,12 +23013,12 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
@@ -23038,22 +23038,22 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M343" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N343" t="n">
@@ -23079,12 +23079,12 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -23104,22 +23104,22 @@
       </c>
       <c r="J344" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>tchr_anna</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
         <is>
-          <t>Teacher Anna</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N344" t="n">
@@ -23145,12 +23145,12 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
+          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
+          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -23170,22 +23170,22 @@
       </c>
       <c r="J345" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K345" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t>tchr_joanna</t>
+          <t>tchr_anna</t>
         </is>
       </c>
       <c r="M345" t="inlineStr">
         <is>
-          <t>Teacher Joanna</t>
+          <t>Teacher Anna</t>
         </is>
       </c>
       <c r="N345" t="n">
@@ -23211,12 +23211,12 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
+          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
+          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -23226,7 +23226,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>Grade 6</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -23236,22 +23236,22 @@
       </c>
       <c r="J346" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K346" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_joanna</t>
         </is>
       </c>
       <c r="M346" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Teacher Joanna</t>
         </is>
       </c>
       <c r="N346" t="n">
@@ -23277,12 +23277,12 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>sec_grade_6_abdullah_ibn_salaam_1st_shift</t>
+          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABDULLAH IBN SALAAM (1ST SHIFT)</t>
+          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -23302,22 +23302,22 @@
       </c>
       <c r="J347" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>tchr_jessa</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
         <is>
-          <t>Teacher Jessa</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N347" t="n">
@@ -23343,22 +23343,22 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
+          <t>sec_grade_6_abdullah_ibn_salaam_1st_shift</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
+          <t>GRADE 6 - ABDULLAH IBN SALAAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>Grade 7</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -23368,22 +23368,22 @@
       </c>
       <c r="J348" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K348" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_jessa</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Jessa</t>
         </is>
       </c>
       <c r="N348" t="n">
@@ -23404,17 +23404,17 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>12:40 PM – 02:50 PM</t>
+          <t>12:40 PM – 01:40 PM</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
+          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
+          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -23434,26 +23434,26 @@
       </c>
       <c r="J349" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K349" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N349" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="350">
@@ -23470,17 +23470,17 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>12:40 PM – 01:40 PM</t>
+          <t>12:40 PM – 02:50 PM</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
+          <t>sec_grade_7_usama_ibn_zayd_1st_shift_girls</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 7 - USAMA IBN ZAYD (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -23490,7 +23490,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>Grade 8</t>
+          <t>Grade 7</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
@@ -23500,26 +23500,26 @@
       </c>
       <c r="J350" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K350" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L350" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="M350" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="N350" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="351">
@@ -23541,12 +23541,12 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
+          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
+          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>Grade 9</t>
+          <t>Grade 8</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
@@ -23566,22 +23566,22 @@
       </c>
       <c r="J351" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K351" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>tchr_raslina</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
         <is>
-          <t>Ustadh Raslina</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="N351" t="n">
@@ -23602,27 +23602,27 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>01:30 PM – 02:30 PM</t>
+          <t>12:40 PM – 01:40 PM</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>sec_kinder_2_abu_bakr_as_sideeq_1st_shift</t>
+          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>Kinder 2 ABU BAKR AS-SIDEEQ (1ST SHIFT)</t>
+          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>Kinder 2</t>
+          <t>Grade 9</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
@@ -23632,22 +23632,22 @@
       </c>
       <c r="J352" t="inlineStr">
         <is>
-          <t>subj_hadith</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K352" t="inlineStr">
         <is>
-          <t>Hadith</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t>tchr_saliha</t>
+          <t>tchr_raslina</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
         <is>
-          <t>Ustadha Saliha</t>
+          <t>Ustadh Raslina</t>
         </is>
       </c>
       <c r="N352" t="n">
@@ -23673,12 +23673,12 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>sec_kinder_2_uthman_ibn_affan_1st_shift</t>
+          <t>sec_kinder_2_abu_bakr_as_sideeq_1st_shift</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Kinder 2 UTHMAN IBN AFFAN (1ST SHIFT)</t>
+          <t>Kinder 2 ABU BAKR AS-SIDEEQ (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -23698,22 +23698,22 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_hadith</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Hadith</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>tchr_abdul_karim</t>
+          <t>tchr_saliha</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
         <is>
-          <t>Alim Abdul Karim</t>
+          <t>Ustadha Saliha</t>
         </is>
       </c>
       <c r="N353" t="n">
@@ -23730,21 +23730,21 @@
         </is>
       </c>
       <c r="C354" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>01:50 PM – 02:50 PM</t>
+          <t>01:30 PM – 02:30 PM</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
+          <t>sec_kinder_2_uthman_ibn_affan_1st_shift</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
+          <t>Kinder 2 UTHMAN IBN AFFAN (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Kinder 2</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -23764,22 +23764,22 @@
       </c>
       <c r="J354" t="inlineStr">
         <is>
-          <t>subj_language</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K354" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_abdul_karim</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Alim Abdul Karim</t>
         </is>
       </c>
       <c r="N354" t="n">
@@ -23805,22 +23805,22 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -23830,22 +23830,22 @@
       </c>
       <c r="J355" t="inlineStr">
         <is>
-          <t>subj_gen_science</t>
+          <t>subj_language</t>
         </is>
       </c>
       <c r="K355" t="inlineStr">
         <is>
-          <t>Gen Science</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N355" t="n">
@@ -23871,12 +23871,12 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>sec_grade_12_abu_musa_al_ashari</t>
+          <t>sec_grade_11_1st_shift_girls</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
+          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -23886,7 +23886,7 @@
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>Grade 12</t>
+          <t>Grade 11</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
@@ -23896,22 +23896,22 @@
       </c>
       <c r="J356" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_gen_science</t>
         </is>
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Gen Science</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="N356" t="n">
@@ -23937,22 +23937,22 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
+          <t>sec_grade_12_abu_musa_al_ashari</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
+          <t>GRADE 12 - ABU MUSA AL-ASHARI</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Senior High School</t>
         </is>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>Grade 2</t>
+          <t>Grade 12</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -23962,22 +23962,22 @@
       </c>
       <c r="J357" t="inlineStr">
         <is>
-          <t>subj_makabansa</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t>Makabansa</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="N357" t="n">
@@ -24003,12 +24003,12 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
+          <t>sec_grade_2_amr_ibn_al_jamuh_1st_shift</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 2 - AMR IBN AL-JAMUH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 2</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
@@ -24028,22 +24028,22 @@
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_makabansa</t>
         </is>
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Makabansa</t>
         </is>
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N358" t="n">
@@ -24069,12 +24069,12 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_3_habib_ibn_zayd_al_ansari_1st_shift_girls</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>Grade 3 - HABIB IBN ZAYD AL-ANSARI (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -24094,22 +24094,22 @@
       </c>
       <c r="J359" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="N359" t="n">
@@ -24135,12 +24135,12 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -24160,22 +24160,22 @@
       </c>
       <c r="J360" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>tchr_silfah</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
         <is>
-          <t>Ustadh Silfah</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N360" t="n">
@@ -24201,12 +24201,12 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -24216,7 +24216,7 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
@@ -24226,22 +24226,22 @@
       </c>
       <c r="J361" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K361" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>tchr_obaydah</t>
+          <t>tchr_silfah</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
         <is>
-          <t>Ustadh Obaydah</t>
+          <t>Ustadh Silfah</t>
         </is>
       </c>
       <c r="N361" t="n">
@@ -24267,12 +24267,12 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -24292,22 +24292,22 @@
       </c>
       <c r="J362" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K362" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_obaydah</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Ustadh Obaydah</t>
         </is>
       </c>
       <c r="N362" t="n">
@@ -24333,12 +24333,12 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -24358,22 +24358,22 @@
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N363" t="n">
@@ -24399,12 +24399,12 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -24414,7 +24414,7 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
@@ -24424,22 +24424,22 @@
       </c>
       <c r="J364" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>tchr_faidh</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
         <is>
-          <t>Ustadh Faidh</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N364" t="n">
@@ -24465,12 +24465,12 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -24490,22 +24490,22 @@
       </c>
       <c r="J365" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_faidh</t>
         </is>
       </c>
       <c r="M365" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Ustadh Faidh</t>
         </is>
       </c>
       <c r="N365" t="n">
@@ -24531,12 +24531,12 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
+          <t>sec_grade_5_hamza_ibn_abdul_1st_shift</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
+          <t>GRADE 5 - HAMZA IBN ABDUL (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -24556,22 +24556,22 @@
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="M366" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="N366" t="n">
@@ -24597,12 +24597,12 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
+          <t>sec_grade_5_muhammad_ibn_maslamah_1st_shift</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
+          <t>GRADE 5 - MUHAMMAD IBN MASLAMAH (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -24612,7 +24612,7 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>Grade 6</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -24622,22 +24622,22 @@
       </c>
       <c r="J367" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K367" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t>tchr_anna</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M367" t="inlineStr">
         <is>
-          <t>Teacher Anna</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N367" t="n">
@@ -24663,22 +24663,22 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
+          <t>sec_grade_6_abbas_ibn_abd_al_muttalib_1st_shift</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
+          <t>GRADE 6 - ABBAS IBN ABD AL-MUTTALIB (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>Grade 7</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -24698,12 +24698,12 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t>tchr_aniah</t>
+          <t>tchr_anna</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
         <is>
-          <t>Teacher Aniah</t>
+          <t>Teacher Anna</t>
         </is>
       </c>
       <c r="N368" t="n">
@@ -24729,12 +24729,12 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
+          <t>sec_grade_7_abu_sufyan_ibn_al_harith_1st_shift_boys</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
+          <t>GRADE 7 - ABU SUFYAN IBN AL-HARITH (1ST SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -24744,7 +24744,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>Grade 8</t>
+          <t>Grade 7</t>
         </is>
       </c>
       <c r="I369" t="inlineStr">
@@ -24754,22 +24754,22 @@
       </c>
       <c r="J369" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K369" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_aniah</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Aniah</t>
         </is>
       </c>
       <c r="N369" t="n">
@@ -24795,12 +24795,12 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
+          <t>sec_grade_8_sa_ad_ibn_mua_dh_1st_shift_girls</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
+          <t>GRADE 8 - SA'AD IBN MUA'DH (1ST SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -24810,7 +24810,7 @@
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>Grade 9</t>
+          <t>Grade 8</t>
         </is>
       </c>
       <c r="I370" t="inlineStr">
@@ -24820,22 +24820,22 @@
       </c>
       <c r="J370" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K370" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>tchr_samsuddin</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M370" t="inlineStr">
         <is>
-          <t>Alim Samsuddin</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N370" t="n">
@@ -24852,31 +24852,31 @@
         </is>
       </c>
       <c r="C371" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>03:10 PM – 04:10 PM</t>
+          <t>01:50 PM – 02:50 PM</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
+          <t>sec_grade_9_abu_hurayrah_1st_shift_girls</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
+          <t>GRADE 9 - ABU HURAYRAH (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>Grade 1</t>
+          <t>Grade 9</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -24886,22 +24886,22 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_samsuddin</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Alim Samsuddin</t>
         </is>
       </c>
       <c r="N371" t="n">
@@ -24918,7 +24918,7 @@
         </is>
       </c>
       <c r="C372" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D372" t="inlineStr">
         <is>
@@ -24927,12 +24927,12 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
+          <t>sec_grade_1_hudhayfah_ibn_al_yam_1st_shift</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
+          <t>GRADE 1 - HUDHAYFAH IBN AL-YAM (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -24947,27 +24947,27 @@
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J372" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K372" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>tchr_abdul_karim</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M372" t="inlineStr">
         <is>
-          <t>Alim Abdul Karim</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N372" t="n">
@@ -24993,22 +24993,22 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
+          <t>sec_grade_1_sa_ad_ibn_abi_waqqaas_2nd_shift</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
+          <t>GRADE 1 - SA'AD IBN ABI WAQQAAS (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>Grade 10</t>
+          <t>Grade 1</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -25018,22 +25018,22 @@
       </c>
       <c r="J373" t="inlineStr">
         <is>
-          <t>subj_mapeh</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
         <is>
-          <t>MAPEH</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_abdul_karim</t>
         </is>
       </c>
       <c r="M373" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Alim Abdul Karim</t>
         </is>
       </c>
       <c r="N373" t="n">
@@ -25050,7 +25050,7 @@
         </is>
       </c>
       <c r="C374" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D374" t="inlineStr">
         <is>
@@ -25059,12 +25059,12 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
+          <t>sec_grade_10_abu_ayyub_al_ansari_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
+          <t>GRADE 10 - ABU AYYUB AL-ANSARI (2ND SHIFT) BOYS</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
@@ -25079,27 +25079,27 @@
       </c>
       <c r="I374" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J374" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_mapeh</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>MAPEH</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="M374" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="N374" t="n">
@@ -25125,22 +25125,22 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>sec_grade_11_1st_shift_girls</t>
+          <t>sec_grade_10_utbah_ibn_ghazwan_1st_shift_girls</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>GRADE 11 (1ST SHIFT GIRLS)</t>
+          <t>GRADE 10 - UTBAH IBN GHAZWAN (1ST SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>Senior High School</t>
+          <t>Junior High School</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>Grade 11</t>
+          <t>Grade 10</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -25150,22 +25150,22 @@
       </c>
       <c r="J375" t="inlineStr">
         <is>
-          <t>subj_mabisang_komunikasyon</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>Mabisang Komunikasyon</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="M375" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="N375" t="n">

</xml_diff>

<commit_message>
fix: transfer Abu Hurayrah Arabic to Hainur
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -22322,12 +22322,12 @@
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="N332" t="n">
@@ -23642,12 +23642,12 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t>tchr_raslina</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
         <is>
-          <t>Ustadh Raslina</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N352" t="n">

</xml_diff>

<commit_message>
fix: assign Khabaab oral exam to Sitti Kauzar
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -8990,12 +8990,12 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_sitti_kauzar</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Teacher Keychelle</t>
+          <t>Teacher Sitti Kauzar</t>
         </is>
       </c>
       <c r="N130" t="n">

</xml_diff>

<commit_message>
fix: restrict replacement proctors to academic teachers
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6229,12 +6229,12 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -45086,12 +45086,12 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R491" t="inlineStr">

</xml_diff>

<commit_message>
fix: exclude principal from automatic proctor coverage
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6229,12 +6229,12 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Franchette</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_ayah</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Ayah</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -45086,12 +45086,12 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_zara</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Zara</t>
         </is>
       </c>
       <c r="R491" t="inlineStr">

</xml_diff>

<commit_message>
fix: cap inactive teacher coverage at two duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -9505,12 +9505,12 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_ayah</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Ayah</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -25157,12 +25157,12 @@
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Franchette</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
@@ -27250,12 +27250,12 @@
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R295" t="inlineStr">
@@ -28797,12 +28797,12 @@
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q312" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R312" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -51638,12 +51638,12 @@
       </c>
       <c r="P563" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q563" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R563" t="inlineStr">
@@ -53640,12 +53640,12 @@
       </c>
       <c r="P585" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q585" t="inlineStr">
         <is>
-          <t>Teacher Keychelle</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R585" t="inlineStr">

</xml_diff>

<commit_message>
fix: assign Wardah in place of Ayah for proctor coverage
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -1042,12 +1042,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -9505,12 +9505,12 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">

</xml_diff>

<commit_message>
fix: merge Franchette and Zara teacher identity
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6229,12 +6229,12 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -15769,7 +15769,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -15789,7 +15789,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -18590,7 +18590,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -18610,7 +18610,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -19591,7 +19591,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N211" t="inlineStr">
@@ -19606,12 +19606,12 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="R211" t="inlineStr">
@@ -20592,7 +20592,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="Q222" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R222" t="inlineStr">
@@ -25157,12 +25157,12 @@
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
@@ -28327,7 +28327,7 @@
       </c>
       <c r="M307" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N307" t="inlineStr">
@@ -28347,7 +28347,7 @@
       </c>
       <c r="Q307" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R307" t="inlineStr">
@@ -31345,12 +31345,12 @@
       </c>
       <c r="P340" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="Q340" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="R340" t="inlineStr">
@@ -34879,7 +34879,7 @@
       </c>
       <c r="M379" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N379" t="inlineStr">
@@ -34894,12 +34894,12 @@
       </c>
       <c r="P379" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q379" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R379" t="inlineStr">
@@ -35076,12 +35076,12 @@
       </c>
       <c r="P381" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q381" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Wendy</t>
         </is>
       </c>
       <c r="R381" t="inlineStr">
@@ -40521,7 +40521,7 @@
       </c>
       <c r="M441" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N441" t="inlineStr">
@@ -40541,7 +40541,7 @@
       </c>
       <c r="Q441" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R441" t="inlineStr">
@@ -45086,12 +45086,12 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_norhaima</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Norhaima</t>
         </is>
       </c>
       <c r="R491" t="inlineStr">
@@ -48347,7 +48347,7 @@
       </c>
       <c r="M527" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N527" t="inlineStr">
@@ -48362,12 +48362,12 @@
       </c>
       <c r="P527" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_ayah</t>
         </is>
       </c>
       <c r="Q527" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Ayah</t>
         </is>
       </c>
       <c r="R527" t="inlineStr">
@@ -49621,7 +49621,7 @@
       </c>
       <c r="M541" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N541" t="inlineStr">
@@ -49641,7 +49641,7 @@
       </c>
       <c r="Q541" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R541" t="inlineStr">
@@ -51896,7 +51896,7 @@
       </c>
       <c r="M566" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N566" t="inlineStr">
@@ -51916,7 +51916,7 @@
       </c>
       <c r="Q566" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R566" t="inlineStr">
@@ -52988,7 +52988,7 @@
       </c>
       <c r="M578" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N578" t="inlineStr">
@@ -53003,12 +53003,12 @@
       </c>
       <c r="P578" t="inlineStr">
         <is>
-          <t>tchr_zara</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q578" t="inlineStr">
         <is>
-          <t>Teacher Zara</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R578" t="inlineStr">
@@ -53898,7 +53898,7 @@
       </c>
       <c r="M588" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="N588" t="inlineStr">
@@ -53918,7 +53918,7 @@
       </c>
       <c r="Q588" t="inlineStr">
         <is>
-          <t>Teacher Franchette</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R588" t="inlineStr">

</xml_diff>

<commit_message>
fix: assign merged identity coverage to Junaisah
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -19606,12 +19606,12 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
-          <t>Teacher Keychelle</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R211" t="inlineStr">
@@ -48362,12 +48362,12 @@
       </c>
       <c r="P527" t="inlineStr">
         <is>
-          <t>tchr_ayah</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q527" t="inlineStr">
         <is>
-          <t>Teacher Ayah</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R527" t="inlineStr">

</xml_diff>

<commit_message>
fix: restore Franchette Zarah proctor duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -25157,12 +25157,12 @@
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
@@ -27250,12 +27250,12 @@
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R295" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -51638,12 +51638,12 @@
       </c>
       <c r="P563" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q563" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R563" t="inlineStr">

</xml_diff>

<commit_message>
fix: rebalance Normylah proctors across six teachers
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -1042,12 +1042,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -6229,12 +6229,12 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -9505,12 +9505,12 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -31345,12 +31345,12 @@
       </c>
       <c r="P340" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_wardah</t>
         </is>
       </c>
       <c r="Q340" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Wardah</t>
         </is>
       </c>
       <c r="R340" t="inlineStr">
@@ -35076,12 +35076,12 @@
       </c>
       <c r="P381" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q381" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R381" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="R434" t="inlineStr">
@@ -45086,12 +45086,12 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>tchr_norhaima</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr">
         <is>
-          <t>Teacher Norhaima</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="R491" t="inlineStr">
@@ -51638,12 +51638,12 @@
       </c>
       <c r="P563" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q563" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R563" t="inlineStr">
@@ -53640,12 +53640,12 @@
       </c>
       <c r="P585" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q585" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R585" t="inlineStr">

</xml_diff>

<commit_message>
fix: standardize Filipino subject labels
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6290,12 +6290,12 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>subj_fil</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>FIL</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -9384,12 +9384,12 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>subj_fil</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -17847,12 +17847,12 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>subj_fil</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>FIL</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L192" t="inlineStr">
@@ -19940,12 +19940,12 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>subj_fil5</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>Fil5</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
@@ -21760,12 +21760,12 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>subj_fil3</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Fil3</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
@@ -25127,12 +25127,12 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>subj_fil</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -35501,12 +35501,12 @@
       </c>
       <c r="J386" t="inlineStr">
         <is>
-          <t>subj_fil4</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t>Fil4</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
@@ -46876,12 +46876,12 @@
       </c>
       <c r="J511" t="inlineStr">
         <is>
-          <t>subj_fil</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K511" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L511" t="inlineStr">

</xml_diff>

<commit_message>
fix: rebalance Junaisah duties and add shift column
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -19606,12 +19606,12 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="R211" t="inlineStr">
@@ -48362,12 +48362,12 @@
       </c>
       <c r="P527" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q527" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Wendy</t>
         </is>
       </c>
       <c r="R527" t="inlineStr">
@@ -53003,12 +53003,12 @@
       </c>
       <c r="P578" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q578" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R578" t="inlineStr">

</xml_diff>

<commit_message>
Correct Franchette exam subject scope
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -4296,34 +4296,30 @@
           <t>Makabansa</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -9756,34 +9752,30 @@
           <t>MAPEH</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -11121,24 +11113,20 @@
           <t>Makabansa</t>
         </is>
       </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -19857,24 +19845,20 @@
           <t>Makabansa</t>
         </is>
       </c>
-      <c r="L214" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P214" t="inlineStr">
@@ -30140,34 +30124,30 @@
           <t>MAPEH</t>
         </is>
       </c>
-      <c r="L327" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L327" t="inlineStr"/>
       <c r="M327" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N327" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O327" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_radzmia</t>
         </is>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Radzmia</t>
         </is>
       </c>
       <c r="R327" t="inlineStr">
@@ -34326,34 +34306,30 @@
           <t>MAPEH</t>
         </is>
       </c>
-      <c r="L373" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L373" t="inlineStr"/>
       <c r="M373" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N373" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O373" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P373" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q373" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R373" t="inlineStr">
@@ -36510,34 +36486,30 @@
           <t>MAPEH</t>
         </is>
       </c>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L397" t="inlineStr"/>
       <c r="M397" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N397" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O397" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P397" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q397" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Wendy</t>
         </is>
       </c>
       <c r="R397" t="inlineStr">
@@ -48795,24 +48767,20 @@
           <t>Makabansa</t>
         </is>
       </c>
-      <c r="L532" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
+      <c r="L532" t="inlineStr"/>
       <c r="M532" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N532" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O532" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P532" t="inlineStr">

</xml_diff>

<commit_message>
Correct Hainur K1 Husain subject scope
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -12383,34 +12383,30 @@
           <t>Qur'an</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>tchr_hainur</t>
-        </is>
-      </c>
+      <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>VACANT_REPLACEMENT_REQUIRED</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>tchr_hainur</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Ustadha Hainur</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">

</xml_diff>

<commit_message>
Accommodate Sophia Anas exam duty
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -11920,22 +11920,22 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>subj_social_studies</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>tchr_shirehan</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>Teacher Shirehan</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -11950,12 +11950,12 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>tchr_shirehan</t>
+          <t>tchr_sophia</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>Teacher Shirehan</t>
+          <t>Teacher Sophia</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -13645,22 +13645,22 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_social_studies</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -13675,12 +13675,12 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>tchr_sophia</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Teacher Sophia</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">

</xml_diff>

<commit_message>
Rebalance Ethel Normylah proctor duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -9770,12 +9770,12 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -25410,12 +25410,12 @@
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
@@ -27503,12 +27503,12 @@
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>tchr_franchette</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr">
         <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R298" t="inlineStr">
@@ -30138,12 +30138,12 @@
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>tchr_radzmia</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>Teacher Radzmia</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R327" t="inlineStr">

</xml_diff>

<commit_message>
Assign Zayd Filipino to Teacher Wendelyn
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -2756,7 +2756,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -14206,7 +14206,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -14226,7 +14226,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -15682,7 +15682,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -35392,22 +35392,22 @@
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>tchr_normylah</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="M385" t="inlineStr">
         <is>
-          <t>Teacher Normylah</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N385" t="inlineStr">
         <is>
-          <t>RESIGNED_INACTIVE</t>
+          <t>ACTIVE_VERIFIED</t>
         </is>
       </c>
       <c r="O385" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="P385" t="inlineStr">
@@ -36500,12 +36500,12 @@
       </c>
       <c r="P397" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_katrina</t>
         </is>
       </c>
       <c r="Q397" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Katrina</t>
         </is>
       </c>
       <c r="R397" t="inlineStr">
@@ -41399,7 +41399,7 @@
       </c>
       <c r="M451" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N451" t="inlineStr">
@@ -41419,7 +41419,7 @@
       </c>
       <c r="Q451" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R451" t="inlineStr">
@@ -48786,7 +48786,7 @@
       </c>
       <c r="Q532" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R532" t="inlineStr">
@@ -52588,7 +52588,7 @@
       </c>
       <c r="M574" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N574" t="inlineStr">
@@ -52608,7 +52608,7 @@
       </c>
       <c r="Q574" t="inlineStr">
         <is>
-          <t>Teacher Wendy</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R574" t="inlineStr">

</xml_diff>

<commit_message>
Assign Ethel to Zayd Filipino proctor duty
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -35412,12 +35412,12 @@
       </c>
       <c r="P385" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q385" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R385" t="inlineStr">
@@ -36955,12 +36955,12 @@
       </c>
       <c r="P402" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_nof</t>
         </is>
       </c>
       <c r="Q402" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Teacher Nof</t>
         </is>
       </c>
       <c r="R402" t="inlineStr">

</xml_diff>

<commit_message>
Remove non-Normylah MAPEH proctor duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -9768,19 +9768,11 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
-        <is>
-          <t>tchr_keychell</t>
-        </is>
-      </c>
-      <c r="Q103" t="inlineStr">
-        <is>
-          <t>Teacher Keychelle</t>
-        </is>
-      </c>
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr"/>
       <c r="R103" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S103" t="n">
@@ -30136,19 +30128,11 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="P327" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
-      <c r="Q327" t="inlineStr">
-        <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
-        </is>
-      </c>
+      <c r="P327" t="inlineStr"/>
+      <c r="Q327" t="inlineStr"/>
       <c r="R327" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S327" t="n">
@@ -34318,19 +34302,11 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="P373" t="inlineStr">
-        <is>
-          <t>tchr_mohaymen</t>
-        </is>
-      </c>
-      <c r="Q373" t="inlineStr">
-        <is>
-          <t>Sir Mohaymen</t>
-        </is>
-      </c>
+      <c r="P373" t="inlineStr"/>
+      <c r="Q373" t="inlineStr"/>
       <c r="R373" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S373" t="n">
@@ -36498,19 +36474,11 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="P397" t="inlineStr">
-        <is>
-          <t>tchr_katrina</t>
-        </is>
-      </c>
-      <c r="Q397" t="inlineStr">
-        <is>
-          <t>Teacher Katrina</t>
-        </is>
-      </c>
+      <c r="P397" t="inlineStr"/>
+      <c r="Q397" t="inlineStr"/>
       <c r="R397" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S397" t="n">
@@ -54239,19 +54207,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="P592" t="inlineStr">
-        <is>
-          <t>tchr_franchette</t>
-        </is>
-      </c>
-      <c r="Q592" t="inlineStr">
-        <is>
-          <t>Teacher Franchette Zarah M. Ranain</t>
-        </is>
-      </c>
+      <c r="P592" t="inlineStr"/>
+      <c r="Q592" t="inlineStr"/>
       <c r="R592" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S592" t="n">

</xml_diff>

<commit_message>
Transfer Dihya proctor duty to Wendelyn
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -27495,12 +27495,12 @@
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R298" t="inlineStr">

</xml_diff>

<commit_message>
Rebalance Wardah and Wendelyn proctor duties
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6316,12 +6316,12 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>tchr_wardah</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Teacher Wardah</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -9592,12 +9592,12 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -12393,12 +12393,12 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>tchr_junaisah</t>
+          <t>tchr_rowena</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Teacher Junaisah</t>
+          <t>Teacher Rowena</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">

</xml_diff>

<commit_message>
Assign Habib Filipino proctor to Franchette
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6316,12 +6316,12 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_franchette</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Franchette Zarah M. Ranain</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">

</xml_diff>

<commit_message>
Assign Junaisah to K1 Husain Quran proctor duty
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -12393,12 +12393,12 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>tchr_rowena</t>
+          <t>tchr_junaisah</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Teacher Rowena</t>
+          <t>Teacher Junaisah</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">

</xml_diff>

<commit_message>
Remove proctor from K1 Husain Quran exam
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -12391,19 +12391,11 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr">
-        <is>
-          <t>tchr_junaisah</t>
-        </is>
-      </c>
-      <c r="Q132" t="inlineStr">
-        <is>
-          <t>Teacher Junaisah</t>
-        </is>
-      </c>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
       <c r="R132" t="inlineStr">
         <is>
-          <t>ACTIVE_ASSIGNED</t>
+          <t>NOT_ASSIGNED</t>
         </is>
       </c>
       <c r="S132" t="n">

</xml_diff>

<commit_message>
Rename K2 oral exams to Circle Time 1
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -5471,12 +5471,12 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -5562,12 +5562,12 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -12545,12 +12545,12 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -14183,12 +14183,12 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -26013,12 +26013,12 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
@@ -42175,12 +42175,12 @@
       </c>
       <c r="J460" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K460" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L460" t="inlineStr">

</xml_diff>

<commit_message>
Rename K1 oral exams to Circle Time 1
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -2741,12 +2741,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -52549,12 +52549,12 @@
       </c>
       <c r="J574" t="inlineStr">
         <is>
-          <t>subj_oral_written_exam</t>
+          <t>subj_circle_time_1</t>
         </is>
       </c>
       <c r="K574" t="inlineStr">
         <is>
-          <t>Oral &amp; Written Exam</t>
+          <t>Circle Time 1</t>
         </is>
       </c>
       <c r="L574" t="inlineStr">

</xml_diff>

<commit_message>
Restore Ethel Grade 7 Anas Math duty
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -35392,12 +35392,12 @@
       </c>
       <c r="P385" t="inlineStr">
         <is>
-          <t>tchr_ethel</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q385" t="inlineStr">
         <is>
-          <t>Teacher Ethel</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R385" t="inlineStr">
@@ -36927,12 +36927,12 @@
       </c>
       <c r="P402" t="inlineStr">
         <is>
-          <t>tchr_nof</t>
+          <t>tchr_ethel</t>
         </is>
       </c>
       <c r="Q402" t="inlineStr">
         <is>
-          <t>Teacher Nof</t>
+          <t>Teacher Ethel</t>
         </is>
       </c>
       <c r="R402" t="inlineStr">

</xml_diff>

<commit_message>
Return Anas Social Studies to Shirehan
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -13758,12 +13758,12 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>tchr_keychell</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Teacher Keychelle</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">

</xml_diff>

<commit_message>
Correct Grade 4 MAPEH teacher assignments
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -27115,12 +27115,12 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
@@ -27135,12 +27135,12 @@
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="Q294" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="R294" t="inlineStr">
@@ -27206,12 +27206,12 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -27226,12 +27226,12 @@
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="R295" t="inlineStr">
@@ -27297,12 +27297,12 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -27317,12 +27317,12 @@
       </c>
       <c r="P296" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q296" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R296" t="inlineStr">
@@ -44915,12 +44915,12 @@
       </c>
       <c r="L490" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M490" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N490" t="inlineStr">
@@ -44935,12 +44935,12 @@
       </c>
       <c r="P490" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="Q490" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="R490" t="inlineStr">
@@ -45006,12 +45006,12 @@
       </c>
       <c r="L491" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M491" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N491" t="inlineStr">
@@ -45026,12 +45026,12 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="R491" t="inlineStr">
@@ -45097,12 +45097,12 @@
       </c>
       <c r="L492" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M492" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N492" t="inlineStr">
@@ -45117,12 +45117,12 @@
       </c>
       <c r="P492" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q492" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R492" t="inlineStr">

</xml_diff>

<commit_message>
Assign Grade 4 F2F MAPEH to Halnaisa
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -1113,12 +1113,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">

</xml_diff>

<commit_message>
Fix merged faculty identities and exam conflicts
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -3934,12 +3934,12 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3954,12 +3954,12 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -5845,12 +5845,12 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -5865,12 +5865,12 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -10486,12 +10486,12 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -10506,12 +10506,12 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -10941,12 +10941,12 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -10961,12 +10961,12 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -14205,12 +14205,12 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -14225,12 +14225,12 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -15297,12 +15297,12 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -15317,12 +15317,12 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -19301,12 +19301,12 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_silfah</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Ustadh Silfah</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
@@ -19321,12 +19321,12 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_bustamante</t>
         </is>
       </c>
       <c r="Q208" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Alim Bustamante</t>
         </is>
       </c>
       <c r="R208" t="inlineStr">
@@ -21303,12 +21303,12 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N230" t="inlineStr">
@@ -21323,12 +21323,12 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q230" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R230" t="inlineStr">
@@ -30130,12 +30130,12 @@
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M327" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N327" t="inlineStr">
@@ -30150,12 +30150,12 @@
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R327" t="inlineStr">
@@ -31040,12 +31040,12 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_hainur</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Ustadha Hainur</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
@@ -31060,12 +31060,12 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_bustamante</t>
         </is>
       </c>
       <c r="Q337" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Alim Bustamante</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">
@@ -37592,12 +37592,12 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N409" t="inlineStr">
@@ -37612,12 +37612,12 @@
       </c>
       <c r="P409" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q409" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R409" t="inlineStr">
@@ -44498,22 +44498,22 @@
       </c>
       <c r="J485" t="inlineStr">
         <is>
-          <t>subj_21st_lit</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K485" t="inlineStr">
         <is>
-          <t>21st Lit.</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L485" t="inlineStr">
         <is>
-          <t>tchr_nof</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M485" t="inlineStr">
         <is>
-          <t>Teacher Nof</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N485" t="inlineStr">
@@ -44528,12 +44528,12 @@
       </c>
       <c r="P485" t="inlineStr">
         <is>
-          <t>tchr_nof</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q485" t="inlineStr">
         <is>
-          <t>Teacher Nof</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R485" t="inlineStr">
@@ -46227,22 +46227,22 @@
       </c>
       <c r="J504" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_21st_lit</t>
         </is>
       </c>
       <c r="K504" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>21st Lit.</t>
         </is>
       </c>
       <c r="L504" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_nof</t>
         </is>
       </c>
       <c r="M504" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Nof</t>
         </is>
       </c>
       <c r="N504" t="inlineStr">
@@ -46257,12 +46257,12 @@
       </c>
       <c r="P504" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_nof</t>
         </is>
       </c>
       <c r="Q504" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Nof</t>
         </is>
       </c>
       <c r="R504" t="inlineStr">
@@ -47784,12 +47784,12 @@
       </c>
       <c r="L521" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M521" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N521" t="inlineStr">
@@ -47804,12 +47804,12 @@
       </c>
       <c r="P521" t="inlineStr">
         <is>
-          <t>tchr_abdulwahab</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q521" t="inlineStr">
         <is>
-          <t>Alim Abdulwahab</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R521" t="inlineStr">

</xml_diff>

<commit_message>
Add missing Grade 6 Dihya MAPEH on Day 4 last period (05:30-06:30 PM)
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S595"/>
+  <dimension ref="A1:S596"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54028,12 +54028,12 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
+          <t>sec_grade_6_dihya_ibn_khalifah_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
+          <t>GRADE 6 - DIHYA IBN KHALIFAH (2ND SHIFT) GIRLS</t>
         </is>
       </c>
       <c r="G590" t="inlineStr">
@@ -54053,42 +54053,42 @@
       </c>
       <c r="J590" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_mapeh</t>
         </is>
       </c>
       <c r="K590" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>MAPEH</t>
         </is>
       </c>
       <c r="L590" t="inlineStr">
         <is>
-          <t>tchr_normylah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M590" t="inlineStr">
         <is>
-          <t>Teacher Normylah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N590" t="inlineStr">
         <is>
-          <t>RESIGNED_INACTIVE</t>
+          <t>ACTIVE_VERIFIED</t>
         </is>
       </c>
       <c r="O590" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="P590" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q590" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R590" t="inlineStr">
@@ -54119,22 +54119,22 @@
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
+          <t>sec_grade_6_khaleed_ibn_waleed_2nd_shift</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
+          <t>GRADE 6 - KHALEED IBN WALEED (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G591" t="inlineStr">
         <is>
-          <t>Junior High School</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="H591" t="inlineStr">
         <is>
-          <t>Grade 7</t>
+          <t>Grade 6</t>
         </is>
       </c>
       <c r="I591" t="inlineStr">
@@ -54144,42 +54144,42 @@
       </c>
       <c r="J591" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K591" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L591" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_normylah</t>
         </is>
       </c>
       <c r="M591" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Teacher Normylah</t>
         </is>
       </c>
       <c r="N591" t="inlineStr">
         <is>
-          <t>ACTIVE_VERIFIED</t>
+          <t>RESIGNED_INACTIVE</t>
         </is>
       </c>
       <c r="O591" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="P591" t="inlineStr">
         <is>
-          <t>tchr_jaisam</t>
+          <t>tchr_mohaymen</t>
         </is>
       </c>
       <c r="Q591" t="inlineStr">
         <is>
-          <t>Ustadh Jaisam</t>
+          <t>Sir Mohaymen</t>
         </is>
       </c>
       <c r="R591" t="inlineStr">
@@ -54210,12 +54210,12 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
+          <t>sec_grade_7_anas_ibn_malik_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
+          <t>GRADE 7 - ANAS IBN MALIK (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G592" t="inlineStr">
@@ -54225,7 +54225,7 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>Grade 8</t>
+          <t>Grade 7</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
@@ -54235,22 +54235,22 @@
       </c>
       <c r="J592" t="inlineStr">
         <is>
-          <t>subj_social_studies</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K592" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L592" t="inlineStr">
         <is>
-          <t>tchr_shirehan</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="M592" t="inlineStr">
         <is>
-          <t>Teacher Shirehan</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="N592" t="inlineStr">
@@ -54265,12 +54265,12 @@
       </c>
       <c r="P592" t="inlineStr">
         <is>
-          <t>tchr_shirehan</t>
+          <t>tchr_jaisam</t>
         </is>
       </c>
       <c r="Q592" t="inlineStr">
         <is>
-          <t>Teacher Shirehan</t>
+          <t>Ustadh Jaisam</t>
         </is>
       </c>
       <c r="R592" t="inlineStr">
@@ -54301,12 +54301,12 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
+          <t>sec_grade_8_mu_adh_ibn_jabal_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
+          <t>GRADE 8 - MU'ADH IBN JABAL (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G593" t="inlineStr">
@@ -54326,22 +54326,22 @@
       </c>
       <c r="J593" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_social_studies</t>
         </is>
       </c>
       <c r="K593" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="L593" t="inlineStr">
         <is>
-          <t>tchr_halnaisa</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="M593" t="inlineStr">
         <is>
-          <t>Teacher Halnaisa</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="N593" t="inlineStr">
@@ -54356,12 +54356,12 @@
       </c>
       <c r="P593" t="inlineStr">
         <is>
-          <t>tchr_halnaisa</t>
+          <t>tchr_shirehan</t>
         </is>
       </c>
       <c r="Q593" t="inlineStr">
         <is>
-          <t>Teacher Halnaisa</t>
+          <t>Teacher Shirehan</t>
         </is>
       </c>
       <c r="R593" t="inlineStr">
@@ -54392,12 +54392,12 @@
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
+          <t>sec_grade_8_nuaym_ibn_mas_ud_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
+          <t>GRADE 8 - NUAYM IBN MAS'UD (2ND SHIFT) MIX</t>
         </is>
       </c>
       <c r="G594" t="inlineStr">
@@ -54407,7 +54407,7 @@
       </c>
       <c r="H594" t="inlineStr">
         <is>
-          <t>Grade 9</t>
+          <t>Grade 8</t>
         </is>
       </c>
       <c r="I594" t="inlineStr">
@@ -54417,22 +54417,22 @@
       </c>
       <c r="J594" t="inlineStr">
         <is>
-          <t>subj_mapeh</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K594" t="inlineStr">
         <is>
-          <t>MAPEH</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L594" t="inlineStr">
         <is>
-          <t>tchr_mohaymen</t>
+          <t>tchr_halnaisa</t>
         </is>
       </c>
       <c r="M594" t="inlineStr">
         <is>
-          <t>Sir Mohaymen</t>
+          <t>Teacher Halnaisa</t>
         </is>
       </c>
       <c r="N594" t="inlineStr">
@@ -54445,11 +54445,19 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="P594" t="inlineStr"/>
-      <c r="Q594" t="inlineStr"/>
+      <c r="P594" t="inlineStr">
+        <is>
+          <t>tchr_halnaisa</t>
+        </is>
+      </c>
+      <c r="Q594" t="inlineStr">
+        <is>
+          <t>Teacher Halnaisa</t>
+        </is>
+      </c>
       <c r="R594" t="inlineStr">
         <is>
-          <t>NOT_ASSIGNED</t>
+          <t>ACTIVE_ASSIGNED</t>
         </is>
       </c>
       <c r="S594" t="n">
@@ -54475,75 +54483,158 @@
       </c>
       <c r="E595" t="inlineStr">
         <is>
+          <t>sec_grade_9_abu_dharr_al_ghifarri_2nd_shift_boys</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>GRADE 9 - ABU DHARR AL GHIFARRI (2ND SHIFT) BOYS</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>Junior High School</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>Grade 9</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>ODL - 2ND SHIFT</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>subj_mapeh</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>MAPEH</t>
+        </is>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>tchr_mohaymen</t>
+        </is>
+      </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>Sir Mohaymen</t>
+        </is>
+      </c>
+      <c r="N595" t="inlineStr">
+        <is>
+          <t>ACTIVE_VERIFIED</t>
+        </is>
+      </c>
+      <c r="O595" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P595" t="inlineStr"/>
+      <c r="Q595" t="inlineStr"/>
+      <c r="R595" t="inlineStr">
+        <is>
+          <t>NOT_ASSIGNED</t>
+        </is>
+      </c>
+      <c r="S595" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="n">
+        <v>4</v>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Monday, September 7, 2026</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>3</v>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>05:30 PM – 06:30 PM</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
           <t>sec_kinder_2_khabaab_ibn_arat_2nd_shift</t>
         </is>
       </c>
-      <c r="F595" t="inlineStr">
+      <c r="F596" t="inlineStr">
         <is>
           <t>Kinder 2 KHABAAB IBN ARAT (2ND SHIFT)</t>
         </is>
       </c>
-      <c r="G595" t="inlineStr">
+      <c r="G596" t="inlineStr">
         <is>
           <t>Elementary</t>
         </is>
       </c>
-      <c r="H595" t="inlineStr">
+      <c r="H596" t="inlineStr">
         <is>
           <t>Kinder 2</t>
         </is>
       </c>
-      <c r="I595" t="inlineStr">
+      <c r="I596" t="inlineStr">
         <is>
           <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
-      <c r="J595" t="inlineStr">
+      <c r="J596" t="inlineStr">
         <is>
           <t>subj_qur_an</t>
         </is>
       </c>
-      <c r="K595" t="inlineStr">
+      <c r="K596" t="inlineStr">
         <is>
           <t>Qur'an</t>
         </is>
       </c>
-      <c r="L595" t="inlineStr">
+      <c r="L596" t="inlineStr">
         <is>
           <t>tchr_faidh</t>
         </is>
       </c>
-      <c r="M595" t="inlineStr">
+      <c r="M596" t="inlineStr">
         <is>
           <t>Ustadh Faidh</t>
         </is>
       </c>
-      <c r="N595" t="inlineStr">
-        <is>
-          <t>ACTIVE_VERIFIED</t>
-        </is>
-      </c>
-      <c r="O595" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="P595" t="inlineStr">
+      <c r="N596" t="inlineStr">
+        <is>
+          <t>ACTIVE_VERIFIED</t>
+        </is>
+      </c>
+      <c r="O596" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P596" t="inlineStr">
         <is>
           <t>tchr_faidh</t>
         </is>
       </c>
-      <c r="Q595" t="inlineStr">
+      <c r="Q596" t="inlineStr">
         <is>
           <t>Ustadh Faidh</t>
         </is>
       </c>
-      <c r="R595" t="inlineStr">
-        <is>
-          <t>ACTIVE_ASSIGNED</t>
-        </is>
-      </c>
-      <c r="S595" t="n">
+      <c r="R596" t="inlineStr">
+        <is>
+          <t>ACTIVE_ASSIGNED</t>
+        </is>
+      </c>
+      <c r="S596" t="n">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Move Grade 9 & 10 Girls F2F Quran to Sunday 8:00 AM - 9:00 AM (Alim Dipatuan)
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -29210,22 +29210,22 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N317" t="inlineStr">
@@ -29240,12 +29240,12 @@
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q317" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R317" t="inlineStr">
@@ -30302,22 +30302,22 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_norhaima</t>
         </is>
       </c>
       <c r="M329" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Norhaima</t>
         </is>
       </c>
       <c r="N329" t="inlineStr">
@@ -30332,12 +30332,12 @@
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_norhaima</t>
         </is>
       </c>
       <c r="Q329" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Norhaima</t>
         </is>
       </c>
       <c r="R329" t="inlineStr">
@@ -31030,22 +31030,22 @@
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>tchr_norhaima</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t>Teacher Norhaima</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
@@ -31060,12 +31060,12 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>tchr_norhaima</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="Q337" t="inlineStr">
         <is>
-          <t>Teacher Norhaima</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">

</xml_diff>

<commit_message>
Move Grade 9 & 10 Girls F2F Quran to Wednesday 8:00 AM (Alim Dipatuan Sunday Madrasah accommodation)
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -1558,22 +1558,22 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>tchr_mamonas</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Alim Mamonas</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -29210,22 +29210,22 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="N317" t="inlineStr">
@@ -29240,12 +29240,12 @@
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_mamonas</t>
         </is>
       </c>
       <c r="Q317" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Alim Mamonas</t>
         </is>
       </c>
       <c r="R317" t="inlineStr">

</xml_diff>

<commit_message>
Completely remove Alim Dipatuan from all Sunday proctor duties (moved to Thursday 12:40 PM)
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -19382,22 +19382,22 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_qur_an</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Qur'an</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="N209" t="inlineStr">
@@ -19412,12 +19412,12 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>tchr_nadzra</t>
+          <t>tchr_dipatuan</t>
         </is>
       </c>
       <c r="Q209" t="inlineStr">
         <is>
-          <t>Teacher Nadzra</t>
+          <t>Alim Dipatuan</t>
         </is>
       </c>
       <c r="R209" t="inlineStr">
@@ -37764,22 +37764,22 @@
       </c>
       <c r="J411" t="inlineStr">
         <is>
-          <t>subj_qur_an</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t>Qur'an</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
@@ -37794,12 +37794,12 @@
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>tchr_dipatuan</t>
+          <t>tchr_nadzra</t>
         </is>
       </c>
       <c r="Q411" t="inlineStr">
         <is>
-          <t>Alim Dipatuan</t>
+          <t>Teacher Nadzra</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">

</xml_diff>

<commit_message>
Restore Grade 3 Salman Al Farsi English exam to Sunday 03:10 PM - 04:10 PM
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6381,12 +6381,12 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -22169,7 +22169,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D240" t="inlineStr">
         <is>
@@ -22178,12 +22178,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -22198,27 +22198,27 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -22233,12 +22233,12 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="Q240" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="R240" t="inlineStr">
@@ -22269,12 +22269,12 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -22294,22 +22294,22 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -22324,12 +22324,12 @@
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
@@ -22351,7 +22351,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -22360,12 +22360,12 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -22380,27 +22380,27 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -22415,12 +22415,12 @@
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="R242" t="inlineStr">
@@ -22451,12 +22451,12 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -22466,7 +22466,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -22486,12 +22486,12 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -22506,12 +22506,12 @@
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="R243" t="inlineStr">
@@ -22533,7 +22533,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -22542,12 +22542,12 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -22562,27 +22562,27 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -22597,12 +22597,12 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
@@ -22624,7 +22624,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
@@ -22633,12 +22633,12 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -22653,27 +22653,27 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -22688,12 +22688,12 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="Q245" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="R245" t="inlineStr">
@@ -22715,7 +22715,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D246" t="inlineStr">
         <is>
@@ -22724,12 +22724,12 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -22744,27 +22744,27 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -22779,12 +22779,12 @@
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="R246" t="inlineStr">
@@ -22806,7 +22806,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D247" t="inlineStr">
         <is>
@@ -22815,12 +22815,12 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -22835,27 +22835,27 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -22870,12 +22870,12 @@
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
@@ -22897,7 +22897,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -22906,12 +22906,12 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -22926,27 +22926,27 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -22961,12 +22961,12 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
@@ -22988,7 +22988,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -22997,12 +22997,12 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -23012,32 +23012,32 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
@@ -23052,12 +23052,12 @@
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
@@ -35546,7 +35546,7 @@
         </is>
       </c>
       <c r="C387" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D387" t="inlineStr">
         <is>
@@ -35555,12 +35555,12 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -35575,27 +35575,27 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t>Teacher Wendelyn</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N387" t="inlineStr">
@@ -35610,12 +35610,12 @@
       </c>
       <c r="P387" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="Q387" t="inlineStr">
         <is>
-          <t>Teacher Wendelyn</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="R387" t="inlineStr">
@@ -35637,7 +35637,7 @@
         </is>
       </c>
       <c r="C388" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
@@ -35646,12 +35646,12 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -35666,27 +35666,27 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
@@ -35701,12 +35701,12 @@
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q388" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R388" t="inlineStr">
@@ -35737,12 +35737,12 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -35752,7 +35752,7 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
@@ -35762,22 +35762,22 @@
       </c>
       <c r="J389" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M389" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N389" t="inlineStr">
@@ -35792,12 +35792,12 @@
       </c>
       <c r="P389" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="Q389" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="R389" t="inlineStr">
@@ -35819,7 +35819,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -35828,12 +35828,12 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -35848,27 +35848,27 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
@@ -35883,12 +35883,12 @@
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="Q390" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="R390" t="inlineStr">
@@ -35919,12 +35919,12 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -35944,22 +35944,22 @@
       </c>
       <c r="J391" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
@@ -35974,12 +35974,12 @@
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="Q391" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="R391" t="inlineStr">
@@ -36001,7 +36001,7 @@
         </is>
       </c>
       <c r="C392" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D392" t="inlineStr">
         <is>
@@ -36010,12 +36010,12 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -36030,7 +36030,7 @@
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
@@ -36045,12 +36045,12 @@
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
@@ -36065,12 +36065,12 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="Q392" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="R392" t="inlineStr">
@@ -36092,7 +36092,7 @@
         </is>
       </c>
       <c r="C393" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -36101,12 +36101,12 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -36121,27 +36121,27 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N393" t="inlineStr">
@@ -36156,12 +36156,12 @@
       </c>
       <c r="P393" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q393" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R393" t="inlineStr">
@@ -36192,12 +36192,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -36207,7 +36207,7 @@
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
@@ -36217,22 +36217,22 @@
       </c>
       <c r="J394" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
         <is>
-          <t>tchr_fhairudz</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>Teacher Fhairudz</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N394" t="inlineStr">
@@ -36247,12 +36247,12 @@
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>tchr_fhairudz</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="Q394" t="inlineStr">
         <is>
-          <t>Teacher Fhairudz</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="R394" t="inlineStr">
@@ -36274,7 +36274,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -36283,12 +36283,12 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -36303,27 +36303,27 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_fhairudz</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Fhairudz</t>
         </is>
       </c>
       <c r="N395" t="inlineStr">
@@ -36338,12 +36338,12 @@
       </c>
       <c r="P395" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_fhairudz</t>
         </is>
       </c>
       <c r="Q395" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Fhairudz</t>
         </is>
       </c>
       <c r="R395" t="inlineStr">

</xml_diff>

<commit_message>
Assign Grade 3 Salman English to Teacher Keychelle on Wed 01:50-02:50 PM matching official poster
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -6381,22 +6381,22 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -6411,12 +6411,12 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_keychell</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Keychelle</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -22169,7 +22169,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D240" t="inlineStr">
         <is>
@@ -22178,12 +22178,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
+          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
+          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -22198,27 +22198,27 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -22233,12 +22233,12 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>tchr_jerlyn</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="Q240" t="inlineStr">
         <is>
-          <t>Teacher Jerlyn</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="R240" t="inlineStr">
@@ -22269,12 +22269,12 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_thabit_ibn_qays_2nd_shift_boys</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 - THABIT IBN QAYS (2ND SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -22294,22 +22294,22 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -22324,12 +22324,12 @@
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_jerlyn</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Teacher Jerlyn</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
@@ -22351,7 +22351,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -22360,12 +22360,12 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -22380,27 +22380,27 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>subj_shaf</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>SHAF</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -22415,12 +22415,12 @@
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>tchr_ersahad</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>Ustadh Ersahad</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="R242" t="inlineStr">
@@ -22451,12 +22451,12 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -22466,7 +22466,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 3</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -22486,12 +22486,12 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -22506,12 +22506,12 @@
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>tchr_abdiraheem</t>
+          <t>tchr_ersahad</t>
         </is>
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>Ustadh Abdiraheem</t>
+          <t>Ustadh Ersahad</t>
         </is>
       </c>
       <c r="R243" t="inlineStr">
@@ -22533,7 +22533,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -22542,12 +22542,12 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -22562,27 +22562,27 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_shaf</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>SHAF</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -22597,12 +22597,12 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_abdiraheem</t>
         </is>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Ustadh Abdiraheem</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
@@ -22624,7 +22624,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
@@ -22633,12 +22633,12 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -22653,27 +22653,27 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -22688,12 +22688,12 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>tchr_arvin</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="Q245" t="inlineStr">
         <is>
-          <t>Teacher Arvin</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="R245" t="inlineStr">
@@ -22715,7 +22715,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D246" t="inlineStr">
         <is>
@@ -22724,12 +22724,12 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_hakim_ibn_hazm_1st_shift</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - HAKIM IBN HAZM(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -22744,27 +22744,27 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>subj_gmrc</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>GMRC</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -22779,12 +22779,12 @@
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>tchr_sahdia</t>
+          <t>tchr_arvin</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
         <is>
-          <t>Teacher Sahdia</t>
+          <t>Teacher Arvin</t>
         </is>
       </c>
       <c r="R246" t="inlineStr">
@@ -22806,7 +22806,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D247" t="inlineStr">
         <is>
@@ -22815,12 +22815,12 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -22835,27 +22835,27 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_gmrc</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>GMRC</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -22870,12 +22870,12 @@
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_sahdia</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Sahdia</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
@@ -22897,7 +22897,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -22906,12 +22906,12 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -22926,27 +22926,27 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -22961,12 +22961,12 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
@@ -22988,7 +22988,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -22997,12 +22997,12 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -23012,32 +23012,32 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>Grade 5</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>subj_tle</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>TLE</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
@@ -23052,12 +23052,12 @@
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
@@ -35546,7 +35546,7 @@
         </is>
       </c>
       <c r="C387" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D387" t="inlineStr">
         <is>
@@ -35555,12 +35555,12 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>sec_grade_3_salman_al_farsi_1st_shift_mix</t>
+          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>GRADE 3 - SALMAN AL FARSI (1ST SHIFT) MIX</t>
+          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -35575,27 +35575,27 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="N387" t="inlineStr">
@@ -35610,12 +35610,12 @@
       </c>
       <c r="P387" t="inlineStr">
         <is>
-          <t>tchr_jenny</t>
+          <t>tchr_wendy</t>
         </is>
       </c>
       <c r="Q387" t="inlineStr">
         <is>
-          <t>Teacher Jenny</t>
+          <t>Teacher Wendelyn</t>
         </is>
       </c>
       <c r="R387" t="inlineStr">
@@ -35637,7 +35637,7 @@
         </is>
       </c>
       <c r="C388" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
@@ -35646,12 +35646,12 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>sec_grade_3_zayd_ibn_haritha_2nd_shift_girls</t>
+          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>GRADE 3 - ZAYD IBN HARITHA (2ND SHIFT) - GIRLS</t>
+          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -35666,27 +35666,27 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_english</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>English</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>Teacher Wendelyn</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
@@ -35701,12 +35701,12 @@
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>tchr_wendy</t>
+          <t>tchr_marham</t>
         </is>
       </c>
       <c r="Q388" t="inlineStr">
         <is>
-          <t>Teacher Wendelyn</t>
+          <t>Teacher Marham</t>
         </is>
       </c>
       <c r="R388" t="inlineStr">
@@ -35737,12 +35737,12 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>sec_grade_3_ammar_ibn_yasir_1st_shift_boys</t>
+          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>GRADE 3 -AMMAR IBN YASIR (1ST SHIFT) - BOYS</t>
+          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -35752,7 +35752,7 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>Grade 3</t>
+          <t>Grade 4</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
@@ -35762,22 +35762,22 @@
       </c>
       <c r="J389" t="inlineStr">
         <is>
-          <t>subj_english</t>
+          <t>subj_arabic</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="M389" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="N389" t="inlineStr">
@@ -35792,12 +35792,12 @@
       </c>
       <c r="P389" t="inlineStr">
         <is>
-          <t>tchr_marham</t>
+          <t>tchr_ali</t>
         </is>
       </c>
       <c r="Q389" t="inlineStr">
         <is>
-          <t>Teacher Marham</t>
+          <t>Ustadh Ali</t>
         </is>
       </c>
       <c r="R389" t="inlineStr">
@@ -35819,7 +35819,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -35828,12 +35828,12 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>sec_grade_4_abdur_rahman_ibn_awf_1st_shift</t>
+          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>GRADE 4 - ABDUR RAHMAN IBN AWF (1ST SHIFT)</t>
+          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -35848,27 +35848,27 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
         <is>
-          <t>subj_arabic</t>
+          <t>subj_araling_panlipunan</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Araling Panlipunan</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
@@ -35883,12 +35883,12 @@
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>tchr_ali</t>
+          <t>tchr_monisa</t>
         </is>
       </c>
       <c r="Q390" t="inlineStr">
         <is>
-          <t>Ustadh Ali</t>
+          <t>Teacher Monisa</t>
         </is>
       </c>
       <c r="R390" t="inlineStr">
@@ -35919,12 +35919,12 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>sec_grade_4_az_zubair_ibn_al_awwaam_2nd_shift</t>
+          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>GRADE 4 - AZ ZUBAIR IBN AL AWWAAM (2ND SHIFT)</t>
+          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -35944,22 +35944,22 @@
       </c>
       <c r="J391" t="inlineStr">
         <is>
-          <t>subj_araling_panlipunan</t>
+          <t>subj_filipino</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t>Araling Panlipunan</t>
+          <t>Filipino</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
@@ -35974,12 +35974,12 @@
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t>tchr_monisa</t>
+          <t>tchr_norhydie</t>
         </is>
       </c>
       <c r="Q391" t="inlineStr">
         <is>
-          <t>Teacher Monisa</t>
+          <t>Teacher Norhydie</t>
         </is>
       </c>
       <c r="R391" t="inlineStr">
@@ -36001,7 +36001,7 @@
         </is>
       </c>
       <c r="C392" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D392" t="inlineStr">
         <is>
@@ -36010,12 +36010,12 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>sec_grade_4_ikrimah_ibn_abi_jahl_2nd_shift</t>
+          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>GRADE 4 - IKRIMAH IBN ABI JAHL (2ND SHIFT)</t>
+          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -36030,7 +36030,7 @@
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
@@ -36045,12 +36045,12 @@
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
@@ -36065,12 +36065,12 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>tchr_norhydie</t>
+          <t>tchr_zuhora</t>
         </is>
       </c>
       <c r="Q392" t="inlineStr">
         <is>
-          <t>Teacher Norhydie</t>
+          <t>Teacher Zuhora</t>
         </is>
       </c>
       <c r="R392" t="inlineStr">
@@ -36092,7 +36092,7 @@
         </is>
       </c>
       <c r="C393" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -36101,12 +36101,12 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>sec_grade_4_usayd_ibn_hudhayr_1st_shift_mix</t>
+          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>GRADE 4 - USAYD IBN HUDHAYR (1ST SHIFT) - MIX</t>
+          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -36121,27 +36121,27 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>ODL - 1ST SHIFT</t>
+          <t>ODL - 2ND SHIFT</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
         <is>
-          <t>subj_filipino</t>
+          <t>subj_science</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t>Filipino</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="N393" t="inlineStr">
@@ -36156,12 +36156,12 @@
       </c>
       <c r="P393" t="inlineStr">
         <is>
-          <t>tchr_zuhora</t>
+          <t>tchr_saimonah</t>
         </is>
       </c>
       <c r="Q393" t="inlineStr">
         <is>
-          <t>Teacher Zuhora</t>
+          <t>Teacher Saimonah</t>
         </is>
       </c>
       <c r="R393" t="inlineStr">
@@ -36192,12 +36192,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>sec_grade_4_hassan_ibn_thabit_2nd_shift_mix</t>
+          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>GRADE 4 -HASSAN IBN THABIT (2ND SHIFT) - MIX</t>
+          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -36207,7 +36207,7 @@
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>Grade 4</t>
+          <t>Grade 5</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
@@ -36217,22 +36217,22 @@
       </c>
       <c r="J394" t="inlineStr">
         <is>
-          <t>subj_science</t>
+          <t>subj_math</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_fhairudz</t>
         </is>
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Fhairudz</t>
         </is>
       </c>
       <c r="N394" t="inlineStr">
@@ -36247,12 +36247,12 @@
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>tchr_saimonah</t>
+          <t>tchr_fhairudz</t>
         </is>
       </c>
       <c r="Q394" t="inlineStr">
         <is>
-          <t>Teacher Saimonah</t>
+          <t>Teacher Fhairudz</t>
         </is>
       </c>
       <c r="R394" t="inlineStr">
@@ -36274,7 +36274,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -36283,12 +36283,12 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>sec_grade_5_al_harith_bin_awf_2nd_shift</t>
+          <t>sec_grade_5_ayyash_ibn_abi_rabi_ah_1st_shift</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>GRADE 5 - AL HARITH BIN AWF (2ND SHIFT)</t>
+          <t>GRADE 5 - AYYASH IBN ABI RABI'AH(1ST SHIFT)</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -36303,27 +36303,27 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>ODL - 2ND SHIFT</t>
+          <t>ODL - 1ST SHIFT</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
         <is>
-          <t>subj_math</t>
+          <t>subj_tle</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>TLE</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>tchr_fhairudz</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
         <is>
-          <t>Teacher Fhairudz</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="N395" t="inlineStr">
@@ -36338,12 +36338,12 @@
       </c>
       <c r="P395" t="inlineStr">
         <is>
-          <t>tchr_fhairudz</t>
+          <t>tchr_jenny</t>
         </is>
       </c>
       <c r="Q395" t="inlineStr">
         <is>
-          <t>Teacher Fhairudz</t>
+          <t>Teacher Jenny</t>
         </is>
       </c>
       <c r="R395" t="inlineStr">

</xml_diff>

<commit_message>
Assign Teacher Aniah as official proctor for Grade 4 Hakim MAPEH (exam_586)
</commit_message>
<xml_diff>
--- a/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
+++ b/Term_Examination_Schedule_S.Y._2026-2027_Optimized.xlsx
@@ -45165,12 +45165,12 @@
       </c>
       <c r="P492" t="inlineStr">
         <is>
-          <t>tchr_halnaisa</t>
+          <t>tchr_aniah</t>
         </is>
       </c>
       <c r="Q492" t="inlineStr">
         <is>
-          <t>Teacher Halnaisa</t>
+          <t>Teacher Aniah</t>
         </is>
       </c>
       <c r="R492" t="inlineStr">

</xml_diff>